<commit_message>
new data for today
</commit_message>
<xml_diff>
--- a/Real Life Stock Test/Stock Test.xlsx
+++ b/Real Life Stock Test/Stock Test.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mofiyinebo/Documents/HybStockAdvisor/Real Life Stock Test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3FBC1D1-ECE7-094A-9544-762EF37650F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2804F691-2CF0-D346-B241-27F3C6DED413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4420" yWindow="900" windowWidth="25820" windowHeight="17180" xr2:uid="{E0FB0739-139A-B84C-896A-CBDE5EAF5D66}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t xml:space="preserve">Date </t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>JOHNHOLT</t>
+  </si>
+  <si>
+    <t>Current Price</t>
   </si>
 </sst>
 </file>
@@ -432,15 +435,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC3B863F-B49F-E946-90E8-9E831B93D1A4}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19.1640625" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="19.1640625" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -456,8 +460,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>46097</v>
       </c>
@@ -474,7 +481,7 @@
         <v>89.8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>46097</v>
       </c>
@@ -491,7 +498,7 @@
         <v>74.400000000000006</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>46097</v>
       </c>
@@ -506,6 +513,12 @@
       </c>
       <c r="E4">
         <v>76.7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <f>J20</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>